<commit_message>
Updated SAU_grids_kan25 model - 2026-07-29 13:09
</commit_message>
<xml_diff>
--- a/VerveStacks_SAU_grids_kan25/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_SAU_grids_kan25/ReportDefs_vervestacks.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_SAU_grids_kan25\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{144B62EE-0DCE-4C33-82B7-796D76AB405C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C1A5D224-8AE5-47C9-B9AD-A5A729B06DF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15952,7 +15952,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A48FA42F-9B31-45F8-A886-29C61EA7C681}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6F49AF5-EDC3-4CC9-930E-C012CA1613DB}">
   <dimension ref="B9:H160"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -18990,7 +18990,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A58C2E98-8B5D-47FC-BAC8-2A2F458D6A75}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79FC8825-53AF-4798-A198-1CE1345A6DA6}">
   <dimension ref="B9:L160"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated SAU_grids_kan25 model - 2026-07-29 14:15
</commit_message>
<xml_diff>
--- a/VerveStacks_SAU_grids_kan25/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_SAU_grids_kan25/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_SAU_grids_kan25\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C1A5D224-8AE5-47C9-B9AD-A5A729B06DF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4895312F-9E9F-4020-9ABF-830EBA33D2D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15952,7 +15952,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6F49AF5-EDC3-4CC9-930E-C012CA1613DB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A23F7D18-6A89-4C30-895A-ECBE42D6D9C4}">
   <dimension ref="B9:H160"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -18990,7 +18990,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79FC8825-53AF-4798-A198-1CE1345A6DA6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22DEBD61-2888-4E04-B50A-80A8659CF324}">
   <dimension ref="B9:L160"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>